<commit_message>
fix: validated 100g calc
</commit_message>
<xml_diff>
--- a/Reporte_GCFID.xlsx
+++ b/Reporte_GCFID.xlsx
@@ -495,7 +495,7 @@
     <col width="11" customWidth="1" min="61" max="61"/>
     <col width="7" customWidth="1" min="62" max="62"/>
     <col width="11" customWidth="1" min="63" max="63"/>
-    <col width="10" customWidth="1" min="64" max="64"/>
+    <col width="11" customWidth="1" min="64" max="64"/>
     <col width="11" customWidth="1" min="65" max="65"/>
     <col width="9" customWidth="1" min="66" max="66"/>
     <col width="12" customWidth="1" min="67" max="67"/>
@@ -531,10 +531,10 @@
     <col width="11" customWidth="1" min="97" max="97"/>
     <col width="9" customWidth="1" min="98" max="98"/>
     <col width="12" customWidth="1" min="99" max="99"/>
-    <col width="9" customWidth="1" min="100" max="100"/>
-    <col width="11" customWidth="1" min="101" max="101"/>
+    <col width="7" customWidth="1" min="100" max="100"/>
+    <col width="7" customWidth="1" min="101" max="101"/>
     <col width="8" customWidth="1" min="102" max="102"/>
-    <col width="8" customWidth="1" min="103" max="103"/>
+    <col width="12" customWidth="1" min="103" max="103"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -855,12 +855,12 @@
       </c>
       <c r="BL1" s="1" t="inlineStr">
         <is>
-          <t>C20:1n11</t>
+          <t>C20:1n11+</t>
         </is>
       </c>
       <c r="BM1" s="1" t="inlineStr">
         <is>
-          <t>C20:1n11</t>
+          <t>C20:1n11+</t>
         </is>
       </c>
       <c r="BN1" s="1" t="inlineStr">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="CV1" s="1" t="inlineStr">
         <is>
-          <t>C24:1n9</t>
+          <t>C24:1</t>
         </is>
       </c>
       <c r="CW1" s="1" t="inlineStr">
         <is>
-          <t>C24:1n9</t>
+          <t>C24:1</t>
         </is>
       </c>
       <c r="CX1" s="1" t="inlineStr">
@@ -1614,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>2.55</v>
+        <v>2.52</v>
       </c>
       <c r="S3" t="n">
         <v>303.655487</v>
@@ -1638,13 +1638,13 @@
         <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>12.02</v>
+        <v>11.9</v>
       </c>
       <c r="AA3" t="n">
         <v>1431.889893</v>
       </c>
       <c r="AB3" t="n">
-        <v>2.77</v>
+        <v>2.74</v>
       </c>
       <c r="AC3" t="n">
         <v>330.036835</v>
@@ -1662,7 +1662,7 @@
         <v>29.714205</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="AI3" t="n">
         <v>36.605503</v>
@@ -1680,13 +1680,13 @@
         <v>62.431286</v>
       </c>
       <c r="AN3" t="n">
-        <v>4.12</v>
+        <v>4.08</v>
       </c>
       <c r="AO3" t="n">
         <v>490.855347</v>
       </c>
       <c r="AP3" t="n">
-        <v>39.89</v>
+        <v>39.52</v>
       </c>
       <c r="AQ3" t="n">
         <v>4753.722656</v>
@@ -1698,13 +1698,13 @@
         <v>0</v>
       </c>
       <c r="AT3" t="n">
-        <v>2.91</v>
+        <v>2.88</v>
       </c>
       <c r="AU3" t="n">
         <v>346.510895</v>
       </c>
       <c r="AV3" t="n">
-        <v>15.05</v>
+        <v>14.91</v>
       </c>
       <c r="AW3" t="n">
         <v>1793.147461</v>
@@ -1722,7 +1722,7 @@
         <v>13.308762</v>
       </c>
       <c r="BB3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="BC3" t="n">
         <v>10.19311</v>
@@ -1734,13 +1734,13 @@
         <v>9.301474000000001</v>
       </c>
       <c r="BF3" t="n">
-        <v>5.52</v>
+        <v>5.47</v>
       </c>
       <c r="BG3" t="n">
         <v>658.304016</v>
       </c>
       <c r="BH3" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="BI3" t="n">
         <v>95.347916</v>
@@ -1752,19 +1752,19 @@
         <v>57.778286</v>
       </c>
       <c r="BL3" t="n">
-        <v>0.44</v>
+        <v>0</v>
       </c>
       <c r="BM3" t="n">
-        <v>52.26635</v>
+        <v>0</v>
       </c>
       <c r="BN3" t="n">
-        <v>1.3</v>
+        <v>1.29</v>
       </c>
       <c r="BO3" t="n">
         <v>154.574692</v>
       </c>
       <c r="BP3" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="BQ3" t="n">
         <v>21.020782</v>
@@ -1794,13 +1794,13 @@
         <v>7.202231</v>
       </c>
       <c r="BZ3" t="n">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="CA3" t="n">
         <v>34.003948</v>
       </c>
       <c r="CB3" t="n">
-        <v>3.89</v>
+        <v>3.85</v>
       </c>
       <c r="CC3" t="n">
         <v>463.404419</v>
@@ -1812,7 +1812,7 @@
         <v>37.0672</v>
       </c>
       <c r="CF3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="CG3" t="n">
         <v>24.549229</v>
@@ -1842,34 +1842,34 @@
         <v>0</v>
       </c>
       <c r="CP3" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="CQ3" t="n">
         <v>78.64299</v>
       </c>
       <c r="CR3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="CS3" t="n">
         <v>23.315809</v>
       </c>
       <c r="CT3" t="n">
-        <v>3.44</v>
+        <v>3.41</v>
       </c>
       <c r="CU3" t="n">
         <v>410.070801</v>
       </c>
       <c r="CV3" t="n">
-        <v>0.32</v>
+        <v>0</v>
       </c>
       <c r="CW3" t="n">
-        <v>38.044754</v>
+        <v>0</v>
       </c>
       <c r="CX3" t="n">
-        <v>0</v>
+        <v>0.84</v>
       </c>
       <c r="CY3" t="n">
-        <v>0</v>
+        <v>111.312909</v>
       </c>
     </row>
     <row r="4">
@@ -1951,13 +1951,13 @@
         <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>13.02</v>
+        <v>12.96</v>
       </c>
       <c r="AA4" t="n">
         <v>1702.834106</v>
       </c>
       <c r="AB4" t="n">
-        <v>2.54</v>
+        <v>2.53</v>
       </c>
       <c r="AC4" t="n">
         <v>331.854675</v>
@@ -1987,19 +1987,19 @@
         <v>9.982901999999999</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="AM4" t="n">
         <v>83.243652</v>
       </c>
       <c r="AN4" t="n">
-        <v>4.38</v>
+        <v>4.36</v>
       </c>
       <c r="AO4" t="n">
         <v>572.2098999999999</v>
       </c>
       <c r="AP4" t="n">
-        <v>36.9</v>
+        <v>36.73</v>
       </c>
       <c r="AQ4" t="n">
         <v>4824.843262</v>
@@ -2011,13 +2011,13 @@
         <v>0</v>
       </c>
       <c r="AT4" t="n">
-        <v>2.71</v>
+        <v>2.7</v>
       </c>
       <c r="AU4" t="n">
         <v>354.177704</v>
       </c>
       <c r="AV4" t="n">
-        <v>20.29</v>
+        <v>20.2</v>
       </c>
       <c r="AW4" t="n">
         <v>2653.434326</v>
@@ -2047,7 +2047,7 @@
         <v>12.987225</v>
       </c>
       <c r="BF4" t="n">
-        <v>5.68</v>
+        <v>5.65</v>
       </c>
       <c r="BG4" t="n">
         <v>742.294189</v>
@@ -2065,13 +2065,13 @@
         <v>58.998814</v>
       </c>
       <c r="BL4" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="BM4" t="n">
-        <v>29.303957</v>
+        <v>0</v>
       </c>
       <c r="BN4" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="BO4" t="n">
         <v>132.799942</v>
@@ -2107,19 +2107,19 @@
         <v>5.638378</v>
       </c>
       <c r="BZ4" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="CA4" t="n">
         <v>29.528717</v>
       </c>
       <c r="CB4" t="n">
-        <v>3.96</v>
+        <v>3.94</v>
       </c>
       <c r="CC4" t="n">
         <v>517.55127</v>
       </c>
       <c r="CD4" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="CE4" t="n">
         <v>41.36441</v>
@@ -2167,22 +2167,22 @@
         <v>28.515562</v>
       </c>
       <c r="CT4" t="n">
-        <v>3.33</v>
+        <v>3.32</v>
       </c>
       <c r="CU4" t="n">
         <v>435.89856</v>
       </c>
       <c r="CV4" t="n">
-        <v>0.28</v>
+        <v>0</v>
       </c>
       <c r="CW4" t="n">
-        <v>37.213444</v>
+        <v>0</v>
       </c>
       <c r="CX4" t="n">
-        <v>0</v>
+        <v>0.43</v>
       </c>
       <c r="CY4" t="n">
-        <v>0</v>
+        <v>61.754053</v>
       </c>
     </row>
     <row r="5">
@@ -2264,7 +2264,7 @@
         <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>11.37</v>
+        <v>11.33</v>
       </c>
       <c r="AA5" t="n">
         <v>1375.357178</v>
@@ -2306,13 +2306,13 @@
         <v>61.940178</v>
       </c>
       <c r="AN5" t="n">
-        <v>3.78</v>
+        <v>3.77</v>
       </c>
       <c r="AO5" t="n">
         <v>457.508789</v>
       </c>
       <c r="AP5" t="n">
-        <v>40.56</v>
+        <v>40.42</v>
       </c>
       <c r="AQ5" t="n">
         <v>4905.338379</v>
@@ -2324,13 +2324,13 @@
         <v>0</v>
       </c>
       <c r="AT5" t="n">
-        <v>2.7</v>
+        <v>2.69</v>
       </c>
       <c r="AU5" t="n">
         <v>326.003937</v>
       </c>
       <c r="AV5" t="n">
-        <v>19.33</v>
+        <v>19.27</v>
       </c>
       <c r="AW5" t="n">
         <v>2338.074951</v>
@@ -2360,31 +2360,31 @@
         <v>9.482535</v>
       </c>
       <c r="BF5" t="n">
-        <v>5.98</v>
+        <v>5.96</v>
       </c>
       <c r="BG5" t="n">
         <v>723.606628</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="BI5" t="n">
         <v>69.64492799999999</v>
       </c>
       <c r="BJ5" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="BK5" t="n">
         <v>56.344971</v>
       </c>
       <c r="BL5" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="BM5" t="n">
-        <v>11.823447</v>
+        <v>0</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="BO5" t="n">
         <v>115.847092</v>
@@ -2426,7 +2426,7 @@
         <v>22.460808</v>
       </c>
       <c r="CB5" t="n">
-        <v>3.17</v>
+        <v>3.16</v>
       </c>
       <c r="CC5" t="n">
         <v>382.947174</v>
@@ -2456,7 +2456,7 @@
         <v>1248.420898</v>
       </c>
       <c r="CL5" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="CM5" t="n">
         <v>18.760756</v>
@@ -2480,22 +2480,22 @@
         <v>23.732975</v>
       </c>
       <c r="CT5" t="n">
-        <v>2.84</v>
+        <v>2.83</v>
       </c>
       <c r="CU5" t="n">
         <v>343.078308</v>
       </c>
       <c r="CV5" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="CW5" t="n">
-        <v>27.794083</v>
+        <v>0</v>
       </c>
       <c r="CX5" t="n">
-        <v>0</v>
+        <v>0.32</v>
       </c>
       <c r="CY5" t="n">
-        <v>0</v>
+        <v>42.216307</v>
       </c>
     </row>
     <row r="6">
@@ -2553,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
       <c r="S6" t="n">
         <v>356.124695</v>
@@ -2577,19 +2577,19 @@
         <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>13.02</v>
+        <v>12.94</v>
       </c>
       <c r="AA6" t="n">
         <v>1854.8927</v>
       </c>
       <c r="AB6" t="n">
-        <v>2.68</v>
+        <v>2.66</v>
       </c>
       <c r="AC6" t="n">
         <v>381.222961</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="AE6" t="n">
         <v>42.098976</v>
@@ -2619,13 +2619,13 @@
         <v>94.411789</v>
       </c>
       <c r="AN6" t="n">
-        <v>4.27</v>
+        <v>4.24</v>
       </c>
       <c r="AO6" t="n">
         <v>607.872253</v>
       </c>
       <c r="AP6" t="n">
-        <v>34.81</v>
+        <v>34.62</v>
       </c>
       <c r="AQ6" t="n">
         <v>4961.315918</v>
@@ -2637,13 +2637,13 @@
         <v>0</v>
       </c>
       <c r="AT6" t="n">
-        <v>2.62</v>
+        <v>2.61</v>
       </c>
       <c r="AU6" t="n">
         <v>373.414246</v>
       </c>
       <c r="AV6" t="n">
-        <v>19.89</v>
+        <v>19.78</v>
       </c>
       <c r="AW6" t="n">
         <v>2834.355225</v>
@@ -2673,7 +2673,7 @@
         <v>9.434416000000001</v>
       </c>
       <c r="BF6" t="n">
-        <v>5.38</v>
+        <v>5.35</v>
       </c>
       <c r="BG6" t="n">
         <v>766.947876</v>
@@ -2691,13 +2691,13 @@
         <v>61.175003</v>
       </c>
       <c r="BL6" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="BM6" t="n">
-        <v>30.935089</v>
+        <v>0</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="BO6" t="n">
         <v>137.999786</v>
@@ -2733,13 +2733,13 @@
         <v>5.707008</v>
       </c>
       <c r="BZ6" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="CA6" t="n">
         <v>35.020016</v>
       </c>
       <c r="CB6" t="n">
-        <v>4.17</v>
+        <v>4.14</v>
       </c>
       <c r="CC6" t="n">
         <v>593.663086</v>
@@ -2793,22 +2793,22 @@
         <v>29.90694</v>
       </c>
       <c r="CT6" t="n">
-        <v>3.5</v>
+        <v>3.48</v>
       </c>
       <c r="CU6" t="n">
         <v>498.49231</v>
       </c>
       <c r="CV6" t="n">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="CW6" t="n">
-        <v>34.856274</v>
+        <v>0</v>
       </c>
       <c r="CX6" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="CY6" t="n">
-        <v>0</v>
+        <v>81.46032</v>
       </c>
     </row>
   </sheetData>
@@ -2858,7 +2858,7 @@
     <col width="9" customWidth="1" min="30" max="30"/>
     <col width="9" customWidth="1" min="31" max="31"/>
     <col width="7" customWidth="1" min="32" max="32"/>
-    <col width="10" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
     <col width="9" customWidth="1" min="34" max="34"/>
     <col width="9" customWidth="1" min="35" max="35"/>
     <col width="9" customWidth="1" min="36" max="36"/>
@@ -2876,7 +2876,7 @@
     <col width="9" customWidth="1" min="48" max="48"/>
     <col width="7" customWidth="1" min="49" max="49"/>
     <col width="9" customWidth="1" min="50" max="50"/>
-    <col width="9" customWidth="1" min="51" max="51"/>
+    <col width="7" customWidth="1" min="51" max="51"/>
     <col width="8" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>C20:1n11</t>
+          <t>C20:1n11+</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="AY1" s="1" t="inlineStr">
         <is>
-          <t>C24:1n9</t>
+          <t>C24:1</t>
         </is>
       </c>
       <c r="AZ1" s="1" t="inlineStr">
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>61.252</v>
+        <v>60.766</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -3242,7 +3242,7 @@
         <v>0.268</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="AH2" t="n">
         <v>0.711</v>
@@ -3293,10 +3293,10 @@
         <v>0.106</v>
       </c>
       <c r="AX2" t="n">
-        <v>1.914</v>
+        <v>1.841</v>
       </c>
       <c r="AY2" t="n">
-        <v>0.172</v>
+        <v>0</v>
       </c>
       <c r="AZ2" t="n">
         <v>0</v>
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71.047</v>
+        <v>70.63800000000001</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -3402,7 +3402,7 @@
         <v>0.293</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.145</v>
+        <v>0</v>
       </c>
       <c r="AH3" t="n">
         <v>0.656</v>
@@ -3453,10 +3453,10 @@
         <v>0.139</v>
       </c>
       <c r="AX3" t="n">
-        <v>2.184</v>
+        <v>2.101</v>
       </c>
       <c r="AY3" t="n">
-        <v>0.181</v>
+        <v>0</v>
       </c>
       <c r="AZ3" t="n">
         <v>0</v>
@@ -3469,7 +3469,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62.895</v>
+        <v>62.651</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -3562,7 +3562,7 @@
         <v>0.265</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="AH4" t="n">
         <v>0.541</v>
@@ -3613,10 +3613,10 @@
         <v>0.11</v>
       </c>
       <c r="AX4" t="n">
-        <v>1.625</v>
+        <v>1.563</v>
       </c>
       <c r="AY4" t="n">
-        <v>0.128</v>
+        <v>0</v>
       </c>
       <c r="AZ4" t="n">
         <v>0</v>
@@ -3629,7 +3629,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.715</v>
+        <v>71.328</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -3722,7 +3722,7 @@
         <v>0.282</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.142</v>
+        <v>0</v>
       </c>
       <c r="AH5" t="n">
         <v>0.631</v>
@@ -3773,10 +3773,10 @@
         <v>0.135</v>
       </c>
       <c r="AX5" t="n">
-        <v>2.313</v>
+        <v>2.225</v>
       </c>
       <c r="AY5" t="n">
-        <v>0.157</v>
+        <v>0</v>
       </c>
       <c r="AZ5" t="n">
         <v>0</v>
@@ -3797,7 +3797,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>61.25151439892343</v>
+        <v>61.17866094978851</v>
       </c>
       <c r="C2" t="n">
         <v>17.20322338013363</v>
@@ -3876,22 +3876,22 @@
         <v>26.57145305455469</v>
       </c>
       <c r="E2" t="n">
-        <v>16.75693847826906</v>
+        <v>16.68408502913413</v>
       </c>
       <c r="F2" t="n">
-        <v>8.10885995936925</v>
+        <v>8.036006510234325</v>
       </c>
       <c r="G2" t="n">
         <v>8.648078518899807</v>
       </c>
       <c r="H2" t="n">
-        <v>1.066497456144563</v>
+        <v>1.076166191240136</v>
       </c>
       <c r="I2" t="n">
         <v>2.099521639503608</v>
       </c>
       <c r="J2" t="n">
-        <v>1.913804067659757</v>
+        <v>1.840950618524833</v>
       </c>
     </row>
     <row r="3">
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71.04696463649425</v>
+        <v>70.96382323203754</v>
       </c>
       <c r="C3" t="n">
         <v>18.34063298897033</v>
@@ -3910,22 +3910,22 @@
         <v>28.66830037666743</v>
       </c>
       <c r="E3" t="n">
-        <v>23.04938756520927</v>
+        <v>22.96624616075256</v>
       </c>
       <c r="F3" t="n">
-        <v>9.498454322418105</v>
+        <v>9.415312917961389</v>
       </c>
       <c r="G3" t="n">
         <v>13.55093324279117</v>
       </c>
       <c r="H3" t="n">
-        <v>1.426646145026825</v>
+        <v>1.439244065583879</v>
       </c>
       <c r="I3" t="n">
         <v>2.517411512382493</v>
       </c>
       <c r="J3" t="n">
-        <v>2.184060740151454</v>
+        <v>2.100919335694738</v>
       </c>
     </row>
     <row r="4">
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62.89542326661402</v>
+        <v>62.8335508356822</v>
       </c>
       <c r="C4" t="n">
         <v>16.6222673706459</v>
@@ -3944,22 +3944,22 @@
         <v>26.76314119080057</v>
       </c>
       <c r="E4" t="n">
-        <v>18.82400597886315</v>
+        <v>18.76213354793133</v>
       </c>
       <c r="F4" t="n">
-        <v>7.569302937869125</v>
+        <v>7.507430506937306</v>
       </c>
       <c r="G4" t="n">
         <v>11.25470304099403</v>
       </c>
       <c r="H4" t="n">
-        <v>1.486887647829088</v>
+        <v>1.499141820972438</v>
       </c>
       <c r="I4" t="n">
         <v>1.761212268143524</v>
       </c>
       <c r="J4" t="n">
-        <v>1.625341166401273</v>
+        <v>1.563468735469453</v>
       </c>
     </row>
     <row r="5">
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.71491990038341</v>
+        <v>71.62687822746356</v>
       </c>
       <c r="C5" t="n">
         <v>20.05175694030636</v>
@@ -3978,22 +3978,22 @@
         <v>27.53049329272156</v>
       </c>
       <c r="E5" t="n">
-        <v>23.14251732912051</v>
+        <v>23.05447565620067</v>
       </c>
       <c r="F5" t="n">
-        <v>9.714174282883317</v>
+        <v>9.626132609963477</v>
       </c>
       <c r="G5" t="n">
         <v>13.4283430462372</v>
       </c>
       <c r="H5" t="n">
-        <v>1.382345287946744</v>
+        <v>1.394988370754238</v>
       </c>
       <c r="I5" t="n">
         <v>2.673860723296452</v>
       </c>
       <c r="J5" t="n">
-        <v>2.312787023240423</v>
+        <v>2.224745350320582</v>
       </c>
     </row>
   </sheetData>
@@ -4007,7 +4007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X193"/>
+  <dimension ref="A1:X197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4227,7 +4227,7 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W2" t="n">
         <v>0</v>
@@ -4305,7 +4305,7 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
@@ -4383,7 +4383,7 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
@@ -4461,7 +4461,7 @@
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
@@ -4539,7 +4539,7 @@
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W6" t="n">
         <v>0</v>
@@ -4617,7 +4617,7 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -4695,7 +4695,7 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
@@ -4773,10 +4773,10 @@
         <v>0.03132810149923027</v>
       </c>
       <c r="V9" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W9" t="n">
-        <v>0.0531370037847823</v>
+        <v>0.0526452556801535</v>
       </c>
       <c r="X9" t="b">
         <v>0</v>
@@ -4851,7 +4851,7 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
@@ -4929,10 +4929,10 @@
         <v>1.467879370822682</v>
       </c>
       <c r="V11" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W11" t="n">
-        <v>2.548115183021703</v>
+        <v>2.524534048927242</v>
       </c>
       <c r="X11" t="b">
         <v>0</v>
@@ -5007,10 +5007,10 @@
         <v>0.01497147838873682</v>
       </c>
       <c r="V12" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W12" t="n">
-        <v>0.0262190528087329</v>
+        <v>0.02597641267839967</v>
       </c>
       <c r="X12" t="b">
         <v>0</v>
@@ -5085,10 +5085,10 @@
         <v>0.1297493925480665</v>
       </c>
       <c r="V13" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W13" t="n">
-        <v>0.227333773762234</v>
+        <v>0.2252299488492134</v>
       </c>
       <c r="X13" t="b">
         <v>0</v>
@@ -5163,7 +5163,7 @@
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W14" t="n">
         <v>0</v>
@@ -5241,10 +5241,10 @@
         <v>6.800793595132538</v>
       </c>
       <c r="V15" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W15" t="n">
-        <v>12.01565764878184</v>
+        <v>11.90446062121535</v>
       </c>
       <c r="X15" t="b">
         <v>0</v>
@@ -5319,10 +5319,10 @@
         <v>1.555267386107386</v>
       </c>
       <c r="V16" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W16" t="n">
-        <v>2.769493407279053</v>
+        <v>2.743863562974556</v>
       </c>
       <c r="X16" t="b">
         <v>0</v>
@@ -5397,10 +5397,10 @@
         <v>0.1588471487189866</v>
       </c>
       <c r="V17" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W17" t="n">
-        <v>0.2828620564360841</v>
+        <v>0.2802443537013339</v>
       </c>
       <c r="X17" t="b">
         <v>0</v>
@@ -5475,10 +5475,10 @@
         <v>0.1401063305728628</v>
       </c>
       <c r="V18" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W18" t="n">
-        <v>0.2493457869152613</v>
+        <v>0.2470382552635072</v>
       </c>
       <c r="X18" t="b">
         <v>0</v>
@@ -5553,10 +5553,10 @@
         <v>0.1697529064344629</v>
       </c>
       <c r="V19" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W19" t="n">
-        <v>0.3071738933125066</v>
+        <v>0.304331200479473</v>
       </c>
       <c r="X19" t="b">
         <v>0</v>
@@ -5631,10 +5631,10 @@
         <v>0.04493783114638336</v>
       </c>
       <c r="V20" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W20" t="n">
-        <v>0.08058016373914187</v>
+        <v>0.0798344471957347</v>
       </c>
       <c r="X20" t="b">
         <v>0</v>
@@ -5709,10 +5709,10 @@
         <v>0.2872046630155305</v>
       </c>
       <c r="V21" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W21" t="n">
-        <v>0.5238901128732482</v>
+        <v>0.5190418536247098</v>
       </c>
       <c r="X21" t="b">
         <v>0</v>
@@ -5787,10 +5787,10 @@
         <v>2.299158610885939</v>
       </c>
       <c r="V22" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W22" t="n">
-        <v>4.11899674084434</v>
+        <v>4.080878128652989</v>
       </c>
       <c r="X22" t="b">
         <v>0</v>
@@ -5865,10 +5865,10 @@
         <v>22.10876172597886</v>
       </c>
       <c r="V23" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W23" t="n">
-        <v>39.8907096773444</v>
+        <v>39.52154733323515</v>
       </c>
       <c r="X23" t="b">
         <v>0</v>
@@ -5943,10 +5943,10 @@
         <v>1.611563686403238</v>
       </c>
       <c r="V24" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W24" t="n">
-        <v>2.907734948598357</v>
+        <v>2.880825769534977</v>
       </c>
       <c r="X24" t="b">
         <v>0</v>
@@ -6021,10 +6021,10 @@
         <v>8.280214057623933</v>
       </c>
       <c r="V25" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W25" t="n">
-        <v>15.04713883105495</v>
+        <v>14.90788743422747</v>
       </c>
       <c r="X25" t="b">
         <v>0</v>
@@ -6099,10 +6099,10 @@
         <v>0.06145584636122332</v>
       </c>
       <c r="V26" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1116800418131545</v>
+        <v>0.1106465163040965</v>
       </c>
       <c r="X26" t="b">
         <v>0</v>
@@ -6177,10 +6177,10 @@
         <v>0.04672627301366389</v>
       </c>
       <c r="V27" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W27" t="n">
-        <v>0.08553514827607854</v>
+        <v>0.08474357660195356</v>
       </c>
       <c r="X27" t="b">
         <v>0</v>
@@ -6255,10 +6255,10 @@
         <v>0.04263892143584909</v>
       </c>
       <c r="V28" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W28" t="n">
-        <v>0.07805301454881514</v>
+        <v>0.07733068511299668</v>
       </c>
       <c r="X28" t="b">
         <v>0</v>
@@ -6333,10 +6333,10 @@
         <v>3.01773400410293</v>
       </c>
       <c r="V29" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W29" t="n">
-        <v>5.524136826047034</v>
+        <v>5.473014564338014</v>
       </c>
       <c r="X29" t="b">
         <v>0</v>
@@ -6411,10 +6411,10 @@
         <v>0.4339297224804607</v>
       </c>
       <c r="V30" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W30" t="n">
-        <v>0.8001089454619356</v>
+        <v>0.7927044621564591</v>
       </c>
       <c r="X30" t="b">
         <v>0</v>
@@ -6489,10 +6489,10 @@
         <v>0.2675660178680626</v>
       </c>
       <c r="V31" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W31" t="n">
-        <v>0.4848446151273548</v>
+        <v>0.4803576963410787</v>
       </c>
       <c r="X31" t="b">
         <v>0</v>
@@ -6567,10 +6567,10 @@
         <v>0.240493604108231</v>
       </c>
       <c r="V32" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W32" t="n">
-        <v>0.4385913811621239</v>
+        <v>0.4345325057075246</v>
       </c>
       <c r="X32" t="b">
         <v>0</v>
@@ -6645,10 +6645,10 @@
         <v>0.7112458565764674</v>
       </c>
       <c r="V33" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W33" t="n">
-        <v>1.297108518700246</v>
+        <v>1.28510463044655</v>
       </c>
       <c r="X33" t="b">
         <v>0</v>
@@ -6723,10 +6723,10 @@
         <v>0.09609107643471639</v>
       </c>
       <c r="V34" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W34" t="n">
-        <v>0.1763952151535299</v>
+        <v>0.1747627931775249</v>
       </c>
       <c r="X34" t="b">
         <v>0</v>
@@ -6801,10 +6801,10 @@
         <v>0.03742997712461711</v>
       </c>
       <c r="V35" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W35" t="n">
-        <v>0.06870477289784027</v>
+        <v>0.06806895530473123</v>
       </c>
       <c r="X35" t="b">
         <v>0</v>
@@ -6879,7 +6879,7 @@
         <v>0</v>
       </c>
       <c r="V36" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W36" t="n">
         <v>0</v>
@@ -6957,10 +6957,10 @@
         <v>0.1876171347028762</v>
       </c>
       <c r="V37" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W37" t="n">
-        <v>0.3448929870525179</v>
+        <v>0.3417012287559875</v>
       </c>
       <c r="X37" t="b">
         <v>0</v>
@@ -7035,10 +7035,10 @@
         <v>0.03292589720857358</v>
       </c>
       <c r="V38" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W38" t="n">
-        <v>0.0604372875420458</v>
+        <v>0.05987798010126347</v>
       </c>
       <c r="X38" t="b">
         <v>0</v>
@@ -7113,10 +7113,10 @@
         <v>0.1540464647033401</v>
       </c>
       <c r="V39" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W39" t="n">
-        <v>0.2853430298908551</v>
+        <v>0.282702367374651</v>
       </c>
       <c r="X39" t="b">
         <v>0</v>
@@ -7191,10 +7191,10 @@
         <v>2.099521639503608</v>
       </c>
       <c r="V40" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W40" t="n">
-        <v>3.88864317000949</v>
+        <v>3.852656328971653</v>
       </c>
       <c r="X40" t="b">
         <v>0</v>
@@ -7269,10 +7269,10 @@
         <v>0.170066367856838</v>
       </c>
       <c r="V41" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W41" t="n">
-        <v>0.3110482055828978</v>
+        <v>0.3081696585318992</v>
       </c>
       <c r="X41" t="b">
         <v>0</v>
@@ -7347,10 +7347,10 @@
         <v>0.1119715293345591</v>
       </c>
       <c r="V42" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W42" t="n">
-        <v>0.2060040571190865</v>
+        <v>0.2040976247382836</v>
       </c>
       <c r="X42" t="b">
         <v>0</v>
@@ -7425,7 +7425,7 @@
         <v>0</v>
       </c>
       <c r="V43" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W43" t="n">
         <v>0</v>
@@ -7503,10 +7503,10 @@
         <v>0.09269438723718565</v>
       </c>
       <c r="V44" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W44" t="n">
-        <v>0.1741533791909382</v>
+        <v>0.1725417039358051</v>
       </c>
       <c r="X44" t="b">
         <v>0</v>
@@ -7581,7 +7581,7 @@
         <v>5.790441261738232</v>
       </c>
       <c r="V45" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W45" t="n">
         <v>0</v>
@@ -7659,10 +7659,10 @@
         <v>0.3642037764733935</v>
       </c>
       <c r="V46" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W46" t="n">
-        <v>0.6599301039583471</v>
+        <v>0.6538228838538152</v>
       </c>
       <c r="X46" t="b">
         <v>0</v>
@@ -7737,10 +7737,10 @@
         <v>0.1061343312091718</v>
       </c>
       <c r="V47" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W47" t="n">
-        <v>0.1956538580256433</v>
+        <v>0.1938432099462539</v>
       </c>
       <c r="X47" t="b">
         <v>0</v>
@@ -7770,7 +7770,7 @@
         <v>13295.46270775795</v>
       </c>
       <c r="G48" t="n">
-        <v>1.0245</v>
+        <v>0.9855</v>
       </c>
       <c r="H48" t="n">
         <v>0.959</v>
@@ -7806,19 +7806,19 @@
         <v>1267.283203125</v>
       </c>
       <c r="S48" t="n">
-        <v>0.0006785123910368276</v>
+        <v>0.0006526832224175634</v>
       </c>
       <c r="T48" t="n">
-        <v>0.0006506933830043176</v>
+        <v>0.0006259232102984433</v>
       </c>
       <c r="U48" t="n">
-        <v>1.913804067659757</v>
+        <v>1.840950618524833</v>
       </c>
       <c r="V48" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W48" t="n">
-        <v>3.441095840880436</v>
+        <v>3.409250756719262</v>
       </c>
       <c r="X48" t="b">
         <v>0</v>
@@ -7893,10 +7893,10 @@
         <v>0.1722399565108213</v>
       </c>
       <c r="V49" t="n">
-        <v>11916.86659550667</v>
+        <v>12028.17950463295</v>
       </c>
       <c r="W49" t="n">
-        <v>0.3192513210030004</v>
+        <v>0.3162968595011942</v>
       </c>
       <c r="X49" t="b">
         <v>0</v>
@@ -7971,7 +7971,7 @@
         <v>0</v>
       </c>
       <c r="V50" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W50" t="n">
         <v>0</v>
@@ -8049,7 +8049,7 @@
         <v>0</v>
       </c>
       <c r="V51" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W51" t="n">
         <v>0</v>
@@ -8127,7 +8127,7 @@
         <v>0</v>
       </c>
       <c r="V52" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W52" t="n">
         <v>0</v>
@@ -8205,7 +8205,7 @@
         <v>0</v>
       </c>
       <c r="V53" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W53" t="n">
         <v>0</v>
@@ -8283,7 +8283,7 @@
         <v>0</v>
       </c>
       <c r="V54" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W54" t="n">
         <v>0</v>
@@ -8361,7 +8361,7 @@
         <v>0</v>
       </c>
       <c r="V55" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W55" t="n">
         <v>0</v>
@@ -8439,7 +8439,7 @@
         <v>0</v>
       </c>
       <c r="V56" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W56" t="n">
         <v>0</v>
@@ -8517,10 +8517,10 @@
         <v>0.03525763271339352</v>
       </c>
       <c r="V57" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W57" t="n">
-        <v>0.05076823743319937</v>
+        <v>0.05052958507828838</v>
       </c>
       <c r="X57" t="b">
         <v>0</v>
@@ -8595,7 +8595,7 @@
         <v>0</v>
       </c>
       <c r="V58" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W58" t="n">
         <v>0</v>
@@ -8673,7 +8673,7 @@
         <v>0</v>
       </c>
       <c r="V59" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W59" t="n">
         <v>0</v>
@@ -8751,10 +8751,10 @@
         <v>0.01386710325718668</v>
       </c>
       <c r="V60" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W60" t="n">
-        <v>0.02061645599234017</v>
+        <v>0.02051954174001923</v>
       </c>
       <c r="X60" t="b">
         <v>0</v>
@@ -8829,10 +8829,10 @@
         <v>0.1467322186360954</v>
       </c>
       <c r="V61" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W61" t="n">
-        <v>0.2182529204264878</v>
+        <v>0.2172269526943105</v>
       </c>
       <c r="X61" t="b">
         <v>0</v>
@@ -8907,7 +8907,7 @@
         <v>0</v>
       </c>
       <c r="V62" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W62" t="n">
         <v>0</v>
@@ -8985,10 +8985,10 @@
         <v>8.682863269312339</v>
       </c>
       <c r="V63" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W63" t="n">
-        <v>13.02347453684209</v>
+        <v>12.96225352495586</v>
       </c>
       <c r="X63" t="b">
         <v>0</v>
@@ -9063,10 +9063,10 @@
         <v>1.678924797120942</v>
       </c>
       <c r="V64" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W64" t="n">
-        <v>2.538063395166545</v>
+        <v>2.526132415546327</v>
       </c>
       <c r="X64" t="b">
         <v>0</v>
@@ -9141,10 +9141,10 @@
         <v>0.1999767704828839</v>
       </c>
       <c r="V65" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W65" t="n">
-        <v>0.3023087882891443</v>
+        <v>0.3008876890372661</v>
       </c>
       <c r="X65" t="b">
         <v>0</v>
@@ -9219,10 +9219,10 @@
         <v>0.1714326621365272</v>
       </c>
       <c r="V66" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W66" t="n">
-        <v>0.2590083684855494</v>
+        <v>0.2577908167207857</v>
       </c>
       <c r="X66" t="b">
         <v>0</v>
@@ -9297,10 +9297,10 @@
         <v>0.229715060743864</v>
       </c>
       <c r="V67" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W67" t="n">
-        <v>0.3528844362426647</v>
+        <v>0.3512255899643876</v>
       </c>
       <c r="X67" t="b">
         <v>0</v>
@@ -9375,10 +9375,10 @@
         <v>0.05015558790384481</v>
       </c>
       <c r="V68" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W68" t="n">
-        <v>0.07635039957798791</v>
+        <v>0.07599149007907813</v>
       </c>
       <c r="X68" t="b">
         <v>0</v>
@@ -9453,10 +9453,10 @@
         <v>0.4111317198241191</v>
       </c>
       <c r="V69" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W69" t="n">
-        <v>0.6366571955242786</v>
+        <v>0.6336643845332959</v>
       </c>
       <c r="X69" t="b">
         <v>0</v>
@@ -9531,10 +9531,10 @@
         <v>2.877474114715442</v>
       </c>
       <c r="V70" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W70" t="n">
-        <v>4.376328282890466</v>
+        <v>4.355755950594124</v>
       </c>
       <c r="X70" t="b">
         <v>0</v>
@@ -9609,10 +9609,10 @@
         <v>24.09097848242786</v>
       </c>
       <c r="V71" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W71" t="n">
-        <v>36.90096593990573</v>
+        <v>36.72750113463971</v>
       </c>
       <c r="X71" t="b">
         <v>0</v>
@@ -9687,10 +9687,10 @@
         <v>1.768448627188221</v>
       </c>
       <c r="V72" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W72" t="n">
-        <v>2.708792530197345</v>
+        <v>2.696058983614257</v>
       </c>
       <c r="X72" t="b">
         <v>0</v>
@@ -9765,10 +9765,10 @@
         <v>13.15450629183386</v>
       </c>
       <c r="V73" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W73" t="n">
-        <v>20.2937762705612</v>
+        <v>20.19837887758732</v>
       </c>
       <c r="X73" t="b">
         <v>0</v>
@@ -9843,10 +9843,10 @@
         <v>0.08390388000830529</v>
       </c>
       <c r="V74" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W74" t="n">
-        <v>0.1294405530200392</v>
+        <v>0.1288320762565932</v>
       </c>
       <c r="X74" t="b">
         <v>0</v>
@@ -9921,10 +9921,10 @@
         <v>0.06154498180147435</v>
       </c>
       <c r="V75" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W75" t="n">
-        <v>0.09564275320843582</v>
+        <v>0.0951931538243052</v>
       </c>
       <c r="X75" t="b">
         <v>0</v>
@@ -9999,10 +9999,10 @@
         <v>0.0639162745880402</v>
       </c>
       <c r="V76" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W76" t="n">
-        <v>0.09932781353556439</v>
+        <v>0.09886089134549204</v>
       </c>
       <c r="X76" t="b">
         <v>0</v>
@@ -10077,10 +10077,10 @@
         <v>3.653180781629844</v>
       </c>
       <c r="V77" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W77" t="n">
-        <v>5.67715283514559</v>
+        <v>5.650465560546391</v>
       </c>
       <c r="X77" t="b">
         <v>0</v>
@@ -10155,10 +10155,10 @@
         <v>0.4669512479304962</v>
       </c>
       <c r="V78" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W78" t="n">
-        <v>0.730932409892235</v>
+        <v>0.7274964280712967</v>
       </c>
       <c r="X78" t="b">
         <v>0</v>
@@ -10233,10 +10233,10 @@
         <v>0.2933257779163868</v>
       </c>
       <c r="V79" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W79" t="n">
-        <v>0.4512298315466051</v>
+        <v>0.4491086812497018</v>
       </c>
       <c r="X79" t="b">
         <v>0</v>
@@ -10311,10 +10311,10 @@
         <v>0.1447599017618761</v>
       </c>
       <c r="V80" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W80" t="n">
-        <v>0.2241200926059137</v>
+        <v>0.2230665443523694</v>
       </c>
       <c r="X80" t="b">
         <v>0</v>
@@ -10389,10 +10389,10 @@
         <v>0.6560242553534916</v>
       </c>
       <c r="V81" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W81" t="n">
-        <v>1.015669498749766</v>
+        <v>1.010895019076194</v>
       </c>
       <c r="X81" t="b">
         <v>0</v>
@@ -10467,10 +10467,10 @@
         <v>0.08750450265636787</v>
       </c>
       <c r="V82" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W82" t="n">
-        <v>0.136367253619851</v>
+        <v>0.1357262156824606</v>
       </c>
       <c r="X82" t="b">
         <v>0</v>
@@ -10545,10 +10545,10 @@
         <v>0.03386189667519174</v>
       </c>
       <c r="V83" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W83" t="n">
-        <v>0.05276604922404781</v>
+        <v>0.05251800551515921</v>
       </c>
       <c r="X83" t="b">
         <v>0</v>
@@ -10623,7 +10623,7 @@
         <v>0</v>
       </c>
       <c r="V84" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W84" t="n">
         <v>0</v>
@@ -10701,10 +10701,10 @@
         <v>0.2135155698242776</v>
       </c>
       <c r="V85" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W85" t="n">
-        <v>0.3332094929563976</v>
+        <v>0.3316431350485152</v>
       </c>
       <c r="X85" t="b">
         <v>0</v>
@@ -10779,10 +10779,10 @@
         <v>0.02767358512930036</v>
       </c>
       <c r="V86" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W86" t="n">
-        <v>0.04312297592616382</v>
+        <v>0.04292026257080871</v>
       </c>
       <c r="X86" t="b">
         <v>0</v>
@@ -10857,10 +10857,10 @@
         <v>0.1436175849338915</v>
       </c>
       <c r="V87" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W87" t="n">
-        <v>0.2258390838154337</v>
+        <v>0.2247774548933265</v>
       </c>
       <c r="X87" t="b">
         <v>0</v>
@@ -10935,10 +10935,10 @@
         <v>2.517411512382493</v>
       </c>
       <c r="V88" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W88" t="n">
-        <v>3.958292680853701</v>
+        <v>3.9396854587504</v>
       </c>
       <c r="X88" t="b">
         <v>0</v>
@@ -11013,10 +11013,10 @@
         <v>0.2037493107613103</v>
       </c>
       <c r="V89" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W89" t="n">
-        <v>0.3163598518152387</v>
+        <v>0.3148727010404193</v>
       </c>
       <c r="X89" t="b">
         <v>0</v>
@@ -11091,10 +11091,10 @@
         <v>0.08426616538236738</v>
       </c>
       <c r="V90" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W90" t="n">
-        <v>0.1316125629416294</v>
+        <v>0.1309938759501179</v>
       </c>
       <c r="X90" t="b">
         <v>0</v>
@@ -11169,7 +11169,7 @@
         <v>0</v>
       </c>
       <c r="V91" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W91" t="n">
         <v>0</v>
@@ -11247,10 +11247,10 @@
         <v>0.1142445242017296</v>
       </c>
       <c r="V92" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W92" t="n">
-        <v>0.1822173861462895</v>
+        <v>0.1813608149807698</v>
       </c>
       <c r="X92" t="b">
         <v>0</v>
@@ -11325,7 +11325,7 @@
         <v>5.790441261738232</v>
       </c>
       <c r="V93" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W93" t="n">
         <v>0</v>
@@ -11403,10 +11403,10 @@
         <v>0.3913143460588962</v>
       </c>
       <c r="V94" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W94" t="n">
-        <v>0.6019427895538094</v>
+        <v>0.5991131647428688</v>
       </c>
       <c r="X94" t="b">
         <v>0</v>
@@ -11481,10 +11481,10 @@
         <v>0.1393567410406082</v>
       </c>
       <c r="V95" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W95" t="n">
-        <v>0.218090355927138</v>
+        <v>0.2170651523814393</v>
       </c>
       <c r="X95" t="b">
         <v>0</v>
@@ -11514,7 +11514,7 @@
         <v>14317.27817702293</v>
       </c>
       <c r="G96" t="n">
-        <v>1.0245</v>
+        <v>0.9855</v>
       </c>
       <c r="H96" t="n">
         <v>0.959</v>
@@ -11550,19 +11550,19 @@
         <v>1180.410400390625</v>
       </c>
       <c r="S96" t="n">
-        <v>0.0007743281039118817</v>
+        <v>0.0007448514850221176</v>
       </c>
       <c r="T96" t="n">
-        <v>0.0007425806516514945</v>
+        <v>0.0007143125741362107</v>
       </c>
       <c r="U96" t="n">
-        <v>2.184060740151454</v>
+        <v>2.100919335694738</v>
       </c>
       <c r="V96" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W96" t="n">
-        <v>3.333803198868702</v>
+        <v>3.318131589523062</v>
       </c>
       <c r="X96" t="b">
         <v>0</v>
@@ -11637,10 +11637,10 @@
         <v>0.18087545627164</v>
       </c>
       <c r="V97" t="n">
-        <v>13075.11372351646</v>
+        <v>13136.86777663231</v>
       </c>
       <c r="W97" t="n">
-        <v>0.2846127731124254</v>
+        <v>0.2832748596457544</v>
       </c>
       <c r="X97" t="b">
         <v>0</v>
@@ -11715,7 +11715,7 @@
         <v>0</v>
       </c>
       <c r="V98" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W98" t="n">
         <v>0</v>
@@ -11793,7 +11793,7 @@
         <v>0</v>
       </c>
       <c r="V99" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W99" t="n">
         <v>0</v>
@@ -11871,7 +11871,7 @@
         <v>0</v>
       </c>
       <c r="V100" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W100" t="n">
         <v>0</v>
@@ -11949,7 +11949,7 @@
         <v>0</v>
       </c>
       <c r="V101" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W101" t="n">
         <v>0</v>
@@ -12027,7 +12027,7 @@
         <v>0</v>
       </c>
       <c r="V102" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W102" t="n">
         <v>0</v>
@@ -12105,7 +12105,7 @@
         <v>0</v>
       </c>
       <c r="V103" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W103" t="n">
         <v>0</v>
@@ -12183,7 +12183,7 @@
         <v>0</v>
       </c>
       <c r="V104" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W104" t="n">
         <v>0</v>
@@ -12261,10 +12261,10 @@
         <v>0.02711362936694573</v>
       </c>
       <c r="V105" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W105" t="n">
-        <v>0.04464388772790048</v>
+        <v>0.04448858083675709</v>
       </c>
       <c r="X105" t="b">
         <v>0</v>
@@ -12339,7 +12339,7 @@
         <v>0</v>
       </c>
       <c r="V106" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W106" t="n">
         <v>0</v>
@@ -12417,10 +12417,10 @@
         <v>1.189795736757955</v>
       </c>
       <c r="V107" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W107" t="n">
-        <v>2.004991168390091</v>
+        <v>1.998016217036605</v>
       </c>
       <c r="X107" t="b">
         <v>0</v>
@@ -12495,10 +12495,10 @@
         <v>0.01046050020924482</v>
       </c>
       <c r="V108" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W108" t="n">
-        <v>0.01778345457897039</v>
+        <v>0.01772158960293419</v>
       </c>
       <c r="X108" t="b">
         <v>0</v>
@@ -12573,10 +12573,10 @@
         <v>0.1104898205725135</v>
       </c>
       <c r="V109" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W109" t="n">
-        <v>0.1879283338378351</v>
+        <v>0.1872745698676361</v>
       </c>
       <c r="X109" t="b">
         <v>0</v>
@@ -12651,7 +12651,7 @@
         <v>0</v>
       </c>
       <c r="V110" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W110" t="n">
         <v>0</v>
@@ -12729,10 +12729,10 @@
         <v>6.630986099718856</v>
       </c>
       <c r="V111" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W111" t="n">
-        <v>11.37306277307565</v>
+        <v>11.33349822993303</v>
       </c>
       <c r="X111" t="b">
         <v>0</v>
@@ -12807,10 +12807,10 @@
         <v>1.222470022476172</v>
       </c>
       <c r="V112" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W112" t="n">
-        <v>2.113220698254562</v>
+        <v>2.105869238656194</v>
       </c>
       <c r="X112" t="b">
         <v>0</v>
@@ -12885,10 +12885,10 @@
         <v>0.135130989369812</v>
       </c>
       <c r="V113" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W113" t="n">
-        <v>0.2335939519674153</v>
+        <v>0.2327813267164275</v>
       </c>
       <c r="X113" t="b">
         <v>0</v>
@@ -12963,10 +12963,10 @@
         <v>0.1320687566544488</v>
       </c>
       <c r="V114" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W114" t="n">
-        <v>0.2281685233942707</v>
+        <v>0.2273747720919397</v>
       </c>
       <c r="X114" t="b">
         <v>0</v>
@@ -13041,10 +13041,10 @@
         <v>0.1642697572521678</v>
       </c>
       <c r="V115" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W115" t="n">
-        <v>0.2885599578056187</v>
+        <v>0.2875561171403881</v>
       </c>
       <c r="X115" t="b">
         <v>0</v>
@@ -13119,10 +13119,10 @@
         <v>0.04159219450523775</v>
       </c>
       <c r="V116" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W116" t="n">
-        <v>0.07240011230704335</v>
+        <v>0.07214824722689239</v>
       </c>
       <c r="X116" t="b">
         <v>0</v>
@@ -13197,10 +13197,10 @@
         <v>0.28925062359316</v>
       </c>
       <c r="V117" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W117" t="n">
-        <v>0.5121938817314486</v>
+        <v>0.5104120647015519</v>
       </c>
       <c r="X117" t="b">
         <v>0</v>
@@ -13275,10 +13275,10 @@
         <v>2.175341759445427</v>
       </c>
       <c r="V118" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W118" t="n">
-        <v>3.783218106159879</v>
+        <v>3.770057069509886</v>
       </c>
       <c r="X118" t="b">
         <v>0</v>
@@ -13353,10 +13353,10 @@
         <v>23.15859450622683</v>
       </c>
       <c r="V119" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W119" t="n">
-        <v>40.56307860215529</v>
+        <v>40.42196800553114</v>
       </c>
       <c r="X119" t="b">
         <v>0</v>
@@ -13431,10 +13431,10 @@
         <v>1.539097284603093</v>
       </c>
       <c r="V120" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W120" t="n">
-        <v>2.695782082756918</v>
+        <v>2.686404012078468</v>
       </c>
       <c r="X120" t="b">
         <v>0</v>
@@ -13509,10 +13509,10 @@
         <v>10.95964876996345</v>
       </c>
       <c r="V121" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W121" t="n">
-        <v>19.33394002540996</v>
+        <v>19.26668122982298</v>
       </c>
       <c r="X121" t="b">
         <v>0</v>
@@ -13587,10 +13587,10 @@
         <v>0.05323165979973064</v>
       </c>
       <c r="V122" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W122" t="n">
-        <v>0.09390608582654891</v>
+        <v>0.09357940589360816</v>
       </c>
       <c r="X122" t="b">
         <v>0</v>
@@ -13665,10 +13665,10 @@
         <v>0.03652668769892424</v>
       </c>
       <c r="V123" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W123" t="n">
-        <v>0.06490903145818018</v>
+        <v>0.06468322630553892</v>
       </c>
       <c r="X123" t="b">
         <v>0</v>
@@ -13743,10 +13743,10 @@
         <v>0.04412569628952496</v>
       </c>
       <c r="V124" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W124" t="n">
-        <v>0.07841270011064359</v>
+        <v>0.0781399184757966</v>
       </c>
       <c r="X124" t="b">
         <v>0</v>
@@ -13821,10 +13821,10 @@
         <v>3.367205615261064</v>
       </c>
       <c r="V125" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W125" t="n">
-        <v>5.983626465357775</v>
+        <v>5.962810661193005</v>
       </c>
       <c r="X125" t="b">
         <v>0</v>
@@ -13899,10 +13899,10 @@
         <v>0.3217439114056822</v>
       </c>
       <c r="V126" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W126" t="n">
-        <v>0.5759057723687291</v>
+        <v>0.5739023147925597</v>
       </c>
       <c r="X126" t="b">
         <v>0</v>
@@ -13977,10 +13977,10 @@
         <v>0.2648708144799937</v>
       </c>
       <c r="V127" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W127" t="n">
-        <v>0.4659261602206947</v>
+        <v>0.4643052990652487</v>
       </c>
       <c r="X127" t="b">
         <v>0</v>
@@ -14055,10 +14055,10 @@
         <v>0.05522530538000993</v>
       </c>
       <c r="V128" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W128" t="n">
-        <v>0.09777009906165991</v>
+        <v>0.09742997702245504</v>
       </c>
       <c r="X128" t="b">
         <v>0</v>
@@ -14133,10 +14133,10 @@
         <v>0.5411020062117484</v>
       </c>
       <c r="V129" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W129" t="n">
-        <v>0.9579593337827921</v>
+        <v>0.9546267905491388</v>
       </c>
       <c r="X129" t="b">
         <v>0</v>
@@ -14211,10 +14211,10 @@
         <v>0.0724599386465388</v>
       </c>
       <c r="V130" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W130" t="n">
-        <v>0.129125813579061</v>
+        <v>0.1286766114666565</v>
       </c>
       <c r="X130" t="b">
         <v>0</v>
@@ -14289,10 +14289,10 @@
         <v>0.02802333779454695</v>
       </c>
       <c r="V131" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W131" t="n">
-        <v>0.04993425508876386</v>
+        <v>0.04976054409910582</v>
       </c>
       <c r="X131" t="b">
         <v>0</v>
@@ -14367,7 +14367,7 @@
         <v>0</v>
       </c>
       <c r="V132" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W132" t="n">
         <v>0</v>
@@ -14445,10 +14445,10 @@
         <v>0.1580443068905683</v>
       </c>
       <c r="V133" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W133" t="n">
-        <v>0.2820344031567636</v>
+        <v>0.2810532635522398</v>
       </c>
       <c r="X133" t="b">
         <v>0</v>
@@ -14523,10 +14523,10 @@
         <v>0.02781882114109917</v>
       </c>
       <c r="V134" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W134" t="n">
-        <v>0.04956983073581799</v>
+        <v>0.04939738750343183</v>
       </c>
       <c r="X134" t="b">
         <v>0</v>
@@ -14601,10 +14601,10 @@
         <v>0.1032905071896588</v>
       </c>
       <c r="V135" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W135" t="n">
-        <v>0.1857322455447673</v>
+        <v>0.1850861213134627</v>
       </c>
       <c r="X135" t="b">
         <v>0</v>
@@ -14679,10 +14679,10 @@
         <v>1.761212268143524</v>
       </c>
       <c r="V136" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W136" t="n">
-        <v>3.166655411411207</v>
+        <v>3.155639269397184</v>
       </c>
       <c r="X136" t="b">
         <v>0</v>
@@ -14757,10 +14757,10 @@
         <v>0.1914939410678184</v>
       </c>
       <c r="V137" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W137" t="n">
-        <v>0.3399974564499508</v>
+        <v>0.3388146753203204</v>
       </c>
       <c r="X137" t="b">
         <v>0</v>
@@ -14835,10 +14835,10 @@
         <v>0.06686607493148032</v>
       </c>
       <c r="V138" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W138" t="n">
-        <v>0.1194222807892461</v>
+        <v>0.1190068352690067</v>
       </c>
       <c r="X138" t="b">
         <v>0</v>
@@ -14913,7 +14913,7 @@
         <v>0</v>
       </c>
       <c r="V139" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W139" t="n">
         <v>0</v>
@@ -14991,10 +14991,10 @@
         <v>0.08505942205228116</v>
       </c>
       <c r="V140" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W140" t="n">
-        <v>0.1551358831501326</v>
+        <v>0.1545961973623787</v>
       </c>
       <c r="X140" t="b">
         <v>0</v>
@@ -15069,7 +15069,7 @@
         <v>5.790441261738232</v>
       </c>
       <c r="V141" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W141" t="n">
         <v>0</v>
@@ -15147,10 +15147,10 @@
         <v>0.2776312262745431</v>
       </c>
       <c r="V142" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W142" t="n">
-        <v>0.4883522281448064</v>
+        <v>0.4866533513176273</v>
       </c>
       <c r="X142" t="b">
         <v>0</v>
@@ -15225,10 +15225,10 @@
         <v>0.1096655508437065</v>
       </c>
       <c r="V143" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W143" t="n">
-        <v>0.1962520128632216</v>
+        <v>0.1955692925279276</v>
       </c>
       <c r="X143" t="b">
         <v>0</v>
@@ -15258,7 +15258,7 @@
         <v>13383.7488424778</v>
       </c>
       <c r="G144" t="n">
-        <v>1.0245</v>
+        <v>0.9855</v>
       </c>
       <c r="H144" t="n">
         <v>0.959</v>
@@ -15294,19 +15294,19 @@
         <v>1248.4208984375</v>
       </c>
       <c r="S144" t="n">
-        <v>0.000576241915095342</v>
+        <v>0.000554305912470922</v>
       </c>
       <c r="T144" t="n">
-        <v>0.0005526159965764329</v>
+        <v>0.0005315793700596142</v>
       </c>
       <c r="U144" t="n">
-        <v>1.625341166401273</v>
+        <v>1.563468735469453</v>
       </c>
       <c r="V144" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W144" t="n">
-        <v>2.836972967699635</v>
+        <v>2.827103723010269</v>
       </c>
       <c r="X144" t="b">
         <v>0</v>
@@ -15381,10 +15381,10 @@
         <v>0.127733296256759</v>
       </c>
       <c r="V145" t="n">
-        <v>12093.1116373539</v>
+        <v>12135.3279440403</v>
       </c>
       <c r="W145" t="n">
-        <v>0.2298340036467505</v>
+        <v>0.2290344584816213</v>
       </c>
       <c r="X145" t="b">
         <v>0</v>
@@ -15459,7 +15459,7 @@
         <v>0</v>
       </c>
       <c r="V146" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W146" t="n">
         <v>0</v>
@@ -15537,7 +15537,7 @@
         <v>0</v>
       </c>
       <c r="V147" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W147" t="n">
         <v>0</v>
@@ -15615,7 +15615,7 @@
         <v>0</v>
       </c>
       <c r="V148" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W148" t="n">
         <v>0</v>
@@ -15693,7 +15693,7 @@
         <v>0</v>
       </c>
       <c r="V149" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W149" t="n">
         <v>0</v>
@@ -15771,7 +15771,7 @@
         <v>0</v>
       </c>
       <c r="V150" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W150" t="n">
         <v>0</v>
@@ -15849,7 +15849,7 @@
         <v>0</v>
       </c>
       <c r="V151" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W151" t="n">
         <v>0</v>
@@ -15927,7 +15927,7 @@
         <v>0</v>
       </c>
       <c r="V152" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W152" t="n">
         <v>0</v>
@@ -16005,10 +16005,10 @@
         <v>0.03784301559737763</v>
       </c>
       <c r="V153" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W153" t="n">
-        <v>0.05399300750023066</v>
+        <v>0.05368612407577231</v>
       </c>
       <c r="X153" t="b">
         <v>0</v>
@@ -16083,7 +16083,7 @@
         <v>0</v>
       </c>
       <c r="V154" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W154" t="n">
         <v>0</v>
@@ -16161,10 +16161,10 @@
         <v>1.7113934919874</v>
       </c>
       <c r="V155" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W155" t="n">
-        <v>2.499006362403009</v>
+        <v>2.484802604069411</v>
       </c>
       <c r="X155" t="b">
         <v>0</v>
@@ -16239,10 +16239,10 @@
         <v>0.01511722935847149</v>
       </c>
       <c r="V156" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W156" t="n">
-        <v>0.02226964581581526</v>
+        <v>0.02214307044085763</v>
       </c>
       <c r="X156" t="b">
         <v>0</v>
@@ -16317,10 +16317,10 @@
         <v>0.1525157690768106</v>
       </c>
       <c r="V157" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W157" t="n">
-        <v>0.2247823329106735</v>
+        <v>0.2235047235446631</v>
       </c>
       <c r="X157" t="b">
         <v>0</v>
@@ -16395,7 +16395,7 @@
         <v>0</v>
       </c>
       <c r="V158" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W158" t="n">
         <v>0</v>
@@ -16473,10 +16473,10 @@
         <v>8.758047876658186</v>
       </c>
       <c r="V159" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W159" t="n">
-        <v>13.01619552570199</v>
+        <v>12.94221456332775</v>
       </c>
       <c r="X159" t="b">
         <v>0</v>
@@ -16551,10 +16551,10 @@
         <v>1.785912819234397</v>
       </c>
       <c r="V160" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W160" t="n">
-        <v>2.675126493453034</v>
+        <v>2.659921710145369</v>
       </c>
       <c r="X160" t="b">
         <v>0</v>
@@ -16629,10 +16629,10 @@
         <v>0.1972208097733651</v>
       </c>
       <c r="V161" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W161" t="n">
-        <v>0.2954178992405479</v>
+        <v>0.2937388141004056</v>
       </c>
       <c r="X161" t="b">
         <v>0</v>
@@ -16707,10 +16707,10 @@
         <v>0.1471052431786683</v>
       </c>
       <c r="V162" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W162" t="n">
-        <v>0.2202222649854393</v>
+        <v>0.2189705739619227</v>
       </c>
       <c r="X162" t="b">
         <v>0</v>
@@ -16785,10 +16785,10 @@
         <v>0.244458604100805</v>
       </c>
       <c r="V163" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W163" t="n">
-        <v>0.3721013178430239</v>
+        <v>0.3699863823735625</v>
       </c>
       <c r="X163" t="b">
         <v>0</v>
@@ -16863,10 +16863,10 @@
         <v>0.04695216842897339</v>
       </c>
       <c r="V164" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W164" t="n">
-        <v>0.07082074468104711</v>
+        <v>0.07041821639717041</v>
       </c>
       <c r="X164" t="b">
         <v>0</v>
@@ -16941,10 +16941,10 @@
         <v>0.4317715134395422</v>
       </c>
       <c r="V165" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W165" t="n">
-        <v>0.6625085670187527</v>
+        <v>0.658743025753454</v>
       </c>
       <c r="X165" t="b">
         <v>0</v>
@@ -17019,10 +17019,10 @@
         <v>2.830520335252978</v>
       </c>
       <c r="V166" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W166" t="n">
-        <v>4.26557509461557</v>
+        <v>4.241330579391738</v>
       </c>
       <c r="X166" t="b">
         <v>0</v>
@@ -17097,10 +17097,10 @@
         <v>22.93855272371256</v>
       </c>
       <c r="V167" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W167" t="n">
-        <v>34.81465965457687</v>
+        <v>34.61678140198828</v>
       </c>
       <c r="X167" t="b">
         <v>0</v>
@@ -17175,10 +17175,10 @@
         <v>1.726473883588791</v>
       </c>
       <c r="V168" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W168" t="n">
-        <v>2.62033099400925</v>
+        <v>2.605437655299558</v>
       </c>
       <c r="X168" t="b">
         <v>0</v>
@@ -17253,10 +17253,10 @@
         <v>13.01123106376803</v>
       </c>
       <c r="V169" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W169" t="n">
-        <v>19.88930237793592</v>
+        <v>19.77625630944636</v>
       </c>
       <c r="X169" t="b">
         <v>0</v>
@@ -17331,10 +17331,10 @@
         <v>0.07370739451526745</v>
       </c>
       <c r="V170" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W170" t="n">
-        <v>0.1126710185853406</v>
+        <v>0.1120306232893288</v>
       </c>
       <c r="X170" t="b">
         <v>0</v>
@@ -17409,10 +17409,10 @@
         <v>0.05505858860952157</v>
       </c>
       <c r="V171" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W171" t="n">
-        <v>0.08478076712602714</v>
+        <v>0.08429889339184536</v>
       </c>
       <c r="X171" t="b">
         <v>0</v>
@@ -17487,10 +17487,10 @@
         <v>0.04299401640599462</v>
       </c>
       <c r="V172" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W172" t="n">
-        <v>0.06620339868463064</v>
+        <v>0.0658271142981935</v>
       </c>
       <c r="X172" t="b">
         <v>0</v>
@@ -17565,10 +17565,10 @@
         <v>3.495093941264613</v>
       </c>
       <c r="V173" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W173" t="n">
-        <v>5.381844195452187</v>
+        <v>5.351255071914393</v>
       </c>
       <c r="X173" t="b">
         <v>0</v>
@@ -17643,10 +17643,10 @@
         <v>0.489758104049783</v>
       </c>
       <c r="V174" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W174" t="n">
-        <v>0.759626584980584</v>
+        <v>0.7553090479790113</v>
       </c>
       <c r="X174" t="b">
         <v>0</v>
@@ -17721,10 +17721,10 @@
         <v>0.281629959642722</v>
       </c>
       <c r="V175" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W175" t="n">
-        <v>0.4292786320865094</v>
+        <v>0.426838714349737</v>
       </c>
       <c r="X175" t="b">
         <v>0</v>
@@ -17799,10 +17799,10 @@
         <v>0.1415048364818862</v>
       </c>
       <c r="V176" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W176" t="n">
-        <v>0.2170784156062846</v>
+        <v>0.2158445934755769</v>
       </c>
       <c r="X176" t="b">
         <v>0</v>
@@ -17877,10 +17877,10 @@
         <v>0.6312455456498149</v>
       </c>
       <c r="V177" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W177" t="n">
-        <v>0.9683752606274162</v>
+        <v>0.9628712457576979</v>
       </c>
       <c r="X177" t="b">
         <v>0</v>
@@ -17955,10 +17955,10 @@
         <v>0.09204740437386395</v>
       </c>
       <c r="V178" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W178" t="n">
-        <v>0.1421359987430906</v>
+        <v>0.1413281315015242</v>
       </c>
       <c r="X178" t="b">
         <v>0</v>
@@ -18033,10 +18033,10 @@
         <v>0.03811418505795589</v>
       </c>
       <c r="V179" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W179" t="n">
-        <v>0.05884950065317672</v>
+        <v>0.05851501407566882</v>
       </c>
       <c r="X179" t="b">
         <v>0</v>
@@ -18111,7 +18111,7 @@
         <v>0</v>
       </c>
       <c r="V180" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W180" t="n">
         <v>0</v>
@@ -18189,10 +18189,10 @@
         <v>0.2318918044278209</v>
       </c>
       <c r="V181" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W181" t="n">
-        <v>0.3585799989798126</v>
+        <v>0.3565419154737452</v>
       </c>
       <c r="X181" t="b">
         <v>0</v>
@@ -18267,10 +18267,10 @@
         <v>0.02593687426947155</v>
       </c>
       <c r="V182" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W182" t="n">
-        <v>0.04004734974502665</v>
+        <v>0.03981973012539012</v>
       </c>
       <c r="X182" t="b">
         <v>0</v>
@@ -18345,10 +18345,10 @@
         <v>0.1577165537281214</v>
       </c>
       <c r="V183" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W183" t="n">
-        <v>0.2457432561095368</v>
+        <v>0.2443465098369363</v>
       </c>
       <c r="X183" t="b">
         <v>0</v>
@@ -18423,10 +18423,10 @@
         <v>2.673860723296452</v>
       </c>
       <c r="V184" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W184" t="n">
-        <v>4.165866199236472</v>
+        <v>4.142188405680491</v>
       </c>
       <c r="X184" t="b">
         <v>0</v>
@@ -18501,10 +18501,10 @@
         <v>0.2069231781961338</v>
       </c>
       <c r="V185" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W185" t="n">
-        <v>0.3183517203958461</v>
+        <v>0.3165422848659423</v>
       </c>
       <c r="X185" t="b">
         <v>0</v>
@@ -18579,10 +18579,10 @@
         <v>0.08785731755604595</v>
       </c>
       <c r="V186" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W186" t="n">
-        <v>0.1359674335544958</v>
+        <v>0.1351946269716464</v>
       </c>
       <c r="X186" t="b">
         <v>0</v>
@@ -18657,7 +18657,7 @@
         <v>0</v>
       </c>
       <c r="V187" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W187" t="n">
         <v>0</v>
@@ -18735,10 +18735,10 @@
         <v>0.1376851877683934</v>
       </c>
       <c r="V188" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W188" t="n">
-        <v>0.2175977929990246</v>
+        <v>0.2163610188506345</v>
       </c>
       <c r="X188" t="b">
         <v>0</v>
@@ -18813,7 +18813,7 @@
         <v>5.790441261738232</v>
       </c>
       <c r="V189" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W189" t="n">
         <v>0</v>
@@ -18891,10 +18891,10 @@
         <v>0.4213358752660602</v>
       </c>
       <c r="V190" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W190" t="n">
-        <v>0.6422006365846619</v>
+        <v>0.6385505207702468</v>
       </c>
       <c r="X190" t="b">
         <v>0</v>
@@ -18969,10 +18969,10 @@
         <v>0.135336808977853</v>
       </c>
       <c r="V191" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W191" t="n">
-        <v>0.2098636673509837</v>
+        <v>0.2086708521349434</v>
       </c>
       <c r="X191" t="b">
         <v>0</v>
@@ -19002,7 +19002,7 @@
         <v>15606.89176893234</v>
       </c>
       <c r="G192" t="n">
-        <v>1.0245</v>
+        <v>0.9855</v>
       </c>
       <c r="H192" t="n">
         <v>0.959</v>
@@ -19038,19 +19038,19 @@
         <v>1274.779663085938</v>
       </c>
       <c r="S192" t="n">
-        <v>0.0008199662021915994</v>
+        <v>0.0007887522618446279</v>
       </c>
       <c r="T192" t="n">
-        <v>0.0007863475879017437</v>
+        <v>0.0007564134191089981</v>
       </c>
       <c r="U192" t="n">
-        <v>2.312787023240423</v>
+        <v>2.224745350320582</v>
       </c>
       <c r="V192" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W192" t="n">
-        <v>3.498031648268788</v>
+        <v>3.478149667605277</v>
       </c>
       <c r="X192" t="b">
         <v>0</v>
@@ -19125,12 +19125,324 @@
         <v>0.1568767687106246</v>
       </c>
       <c r="V193" t="n">
-        <v>14250.65178632736</v>
+        <v>14332.11210584641</v>
       </c>
       <c r="W193" t="n">
-        <v>0.2445942415389416</v>
+        <v>0.243204025992124</v>
       </c>
       <c r="X193" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Unknow</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>111.3129091262817</v>
+      </c>
+      <c r="C194" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" t="b">
+        <v>0</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>VIT25-7118</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>13295.46270775795</v>
+      </c>
+      <c r="G194" t="n">
+        <v>1.0207</v>
+      </c>
+      <c r="H194" t="n">
+        <v>0.9524</v>
+      </c>
+      <c r="I194" t="n">
+        <v>0.69663</v>
+      </c>
+      <c r="J194" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K194" t="n">
+        <v>10</v>
+      </c>
+      <c r="L194" t="n">
+        <v>0.0960144</v>
+      </c>
+      <c r="M194" t="n">
+        <v>6.966299999999999</v>
+      </c>
+      <c r="N194" t="n">
+        <v>0.01364486972998579</v>
+      </c>
+      <c r="O194" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="P194" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>0.002046730459497868</v>
+      </c>
+      <c r="R194" t="n">
+        <v>1267.283203125</v>
+      </c>
+      <c r="S194" t="n">
+        <v>0</v>
+      </c>
+      <c r="T194" t="n">
+        <v>0</v>
+      </c>
+      <c r="U194" t="n">
+        <v>0</v>
+      </c>
+      <c r="V194" t="n">
+        <v>12028.17950463295</v>
+      </c>
+      <c r="W194" t="n">
+        <v>0.8372247854249508</v>
+      </c>
+      <c r="X194" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Unknow</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>61.75405311584473</v>
+      </c>
+      <c r="C195" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" t="b">
+        <v>0</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>VIT25-7248</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>14317.27817702293</v>
+      </c>
+      <c r="G195" t="n">
+        <v>1.0207</v>
+      </c>
+      <c r="H195" t="n">
+        <v>0.9524</v>
+      </c>
+      <c r="I195" t="n">
+        <v>0.69663</v>
+      </c>
+      <c r="J195" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K195" t="n">
+        <v>10</v>
+      </c>
+      <c r="L195" t="n">
+        <v>0.0960144</v>
+      </c>
+      <c r="M195" t="n">
+        <v>6.966299999999999</v>
+      </c>
+      <c r="N195" t="n">
+        <v>0.01364486972998579</v>
+      </c>
+      <c r="O195" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="P195" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>0.002046730459497868</v>
+      </c>
+      <c r="R195" t="n">
+        <v>1180.410400390625</v>
+      </c>
+      <c r="S195" t="n">
+        <v>0</v>
+      </c>
+      <c r="T195" t="n">
+        <v>0</v>
+      </c>
+      <c r="U195" t="n">
+        <v>0</v>
+      </c>
+      <c r="V195" t="n">
+        <v>13136.86777663231</v>
+      </c>
+      <c r="W195" t="n">
+        <v>0.4313253703134023</v>
+      </c>
+      <c r="X195" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Unknow</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>42.21630668640137</v>
+      </c>
+      <c r="C196" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" t="b">
+        <v>0</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>VIT25-7249</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>13383.7488424778</v>
+      </c>
+      <c r="G196" t="n">
+        <v>1.0207</v>
+      </c>
+      <c r="H196" t="n">
+        <v>0.9524</v>
+      </c>
+      <c r="I196" t="n">
+        <v>0.69663</v>
+      </c>
+      <c r="J196" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K196" t="n">
+        <v>10</v>
+      </c>
+      <c r="L196" t="n">
+        <v>0.0960144</v>
+      </c>
+      <c r="M196" t="n">
+        <v>6.966299999999999</v>
+      </c>
+      <c r="N196" t="n">
+        <v>0.01364486972998579</v>
+      </c>
+      <c r="O196" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="P196" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>0.002046730459497868</v>
+      </c>
+      <c r="R196" t="n">
+        <v>1248.4208984375</v>
+      </c>
+      <c r="S196" t="n">
+        <v>0</v>
+      </c>
+      <c r="T196" t="n">
+        <v>0</v>
+      </c>
+      <c r="U196" t="n">
+        <v>0</v>
+      </c>
+      <c r="V196" t="n">
+        <v>12135.3279440403</v>
+      </c>
+      <c r="W196" t="n">
+        <v>0.3154296093215265</v>
+      </c>
+      <c r="X196" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Unknow</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>81.46031951904479</v>
+      </c>
+      <c r="C197" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" t="b">
+        <v>0</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>VIT25-7250</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>15606.89176893234</v>
+      </c>
+      <c r="G197" t="n">
+        <v>1.0207</v>
+      </c>
+      <c r="H197" t="n">
+        <v>0.9524</v>
+      </c>
+      <c r="I197" t="n">
+        <v>0.69663</v>
+      </c>
+      <c r="J197" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K197" t="n">
+        <v>10</v>
+      </c>
+      <c r="L197" t="n">
+        <v>0.0960144</v>
+      </c>
+      <c r="M197" t="n">
+        <v>6.966299999999999</v>
+      </c>
+      <c r="N197" t="n">
+        <v>0.01364486972998579</v>
+      </c>
+      <c r="O197" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="P197" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>0.002046730459497868</v>
+      </c>
+      <c r="R197" t="n">
+        <v>1274.779663085938</v>
+      </c>
+      <c r="S197" t="n">
+        <v>0</v>
+      </c>
+      <c r="T197" t="n">
+        <v>0</v>
+      </c>
+      <c r="U197" t="n">
+        <v>0</v>
+      </c>
+      <c r="V197" t="n">
+        <v>14332.11210584641</v>
+      </c>
+      <c r="W197" t="n">
+        <v>0.5219509478575475</v>
+      </c>
+      <c r="X197" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>